<commit_message>
atualizei os dados de 2Q26 da NRG
</commit_message>
<xml_diff>
--- a/analise_eua/energia_eletrica/nrg/nrg_indicators.xlsx
+++ b/analise_eua/energia_eletrica/nrg/nrg_indicators.xlsx
@@ -609,10 +609,10 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>15826</v>
+        <v>15770</v>
       </c>
       <c r="H2" t="n">
-        <v>30860700000</v>
+        <v>30751500000</v>
       </c>
       <c r="I2" t="n">
         <v>16622</v>
@@ -630,7 +630,7 @@
         <v>7.07</v>
       </c>
       <c r="N2" t="n">
-        <v>11263.26</v>
+        <v>11223.42</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -691,13 +691,13 @@
         <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>16.2</v>
+        <v>16.14</v>
       </c>
       <c r="C3" t="n">
-        <v>16.2</v>
+        <v>16.14</v>
       </c>
       <c r="D3" t="n">
-        <v>6.17</v>
+        <v>6.19</v>
       </c>
       <c r="E3" t="n">
         <v>3495</v>
@@ -706,10 +706,10 @@
         <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>7.35</v>
+        <v>7.33</v>
       </c>
       <c r="H3" t="n">
-        <v>18222760</v>
+        <v>18158900</v>
       </c>
       <c r="I3" t="n">
         <v>10991</v>
@@ -727,7 +727,7 @@
         <v>4.04</v>
       </c>
       <c r="N3" t="n">
-        <v>8.08</v>
+        <v>8.06</v>
       </c>
       <c r="O3" t="n">
         <v>45.4</v>
@@ -786,7 +786,7 @@
         <v>2023</v>
       </c>
       <c r="B4" t="n">
-        <v>-55.91</v>
+        <v>-55.71</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -801,10 +801,10 @@
         <v>-0.7</v>
       </c>
       <c r="G4" t="n">
-        <v>3.88</v>
+        <v>3.87</v>
       </c>
       <c r="H4" t="n">
-        <v>11292840</v>
+        <v>11254080</v>
       </c>
       <c r="I4" t="n">
         <v>10971</v>
@@ -822,7 +822,7 @@
         <v>3.58</v>
       </c>
       <c r="N4" t="n">
-        <v>14.36</v>
+        <v>14.33</v>
       </c>
       <c r="O4" t="n">
         <v>-6.95</v>
@@ -887,7 +887,7 @@
         <v>0.01</v>
       </c>
       <c r="D5" t="n">
-        <v>17687.97</v>
+        <v>17754.74</v>
       </c>
       <c r="E5" t="n">
         <v>2652</v>
@@ -899,7 +899,7 @@
         <v>1.8</v>
       </c>
       <c r="H5" t="n">
-        <v>6903000</v>
+        <v>6877040</v>
       </c>
       <c r="I5" t="n">
         <v>8302</v>
@@ -917,7 +917,7 @@
         <v>2.05</v>
       </c>
       <c r="N5" t="n">
-        <v>5.56</v>
+        <v>5.55</v>
       </c>
       <c r="O5" t="n">
         <v>31896.55</v>
@@ -976,13 +976,13 @@
         <v>2021</v>
       </c>
       <c r="B6" t="n">
-        <v>4.28</v>
+        <v>4.27</v>
       </c>
       <c r="C6" t="n">
-        <v>4.28</v>
+        <v>4.26</v>
       </c>
       <c r="D6" t="n">
-        <v>23.37</v>
+        <v>23.45</v>
       </c>
       <c r="E6" t="n">
         <v>4126</v>
@@ -991,10 +991,10 @@
         <v>8.1</v>
       </c>
       <c r="G6" t="n">
-        <v>2.6</v>
+        <v>2.59</v>
       </c>
       <c r="H6" t="n">
-        <v>9361450</v>
+        <v>9329600</v>
       </c>
       <c r="I6" t="n">
         <v>8287</v>
@@ -1071,13 +1071,13 @@
         <v>2020</v>
       </c>
       <c r="B7" t="n">
-        <v>15.49</v>
+        <v>15.43</v>
       </c>
       <c r="C7" t="n">
-        <v>15.5</v>
+        <v>15.44</v>
       </c>
       <c r="D7" t="n">
-        <v>6.45</v>
+        <v>6.48</v>
       </c>
       <c r="E7" t="n">
         <v>1540</v>
@@ -1086,10 +1086,10 @@
         <v>5.61</v>
       </c>
       <c r="G7" t="n">
-        <v>4.7</v>
+        <v>4.68</v>
       </c>
       <c r="H7" t="n">
-        <v>7898800</v>
+        <v>7869400</v>
       </c>
       <c r="I7" t="n">
         <v>9039</v>
@@ -1107,7 +1107,7 @@
         <v>3.05</v>
       </c>
       <c r="N7" t="n">
-        <v>8.460000000000001</v>
+        <v>8.44</v>
       </c>
       <c r="O7" t="n">
         <v>30.36</v>
@@ -1172,7 +1172,7 @@
         <v>1.94</v>
       </c>
       <c r="D8" t="n">
-        <v>51.43</v>
+        <v>51.6</v>
       </c>
       <c r="E8" t="n">
         <v>1663</v>
@@ -1181,10 +1181,10 @@
         <v>45.19</v>
       </c>
       <c r="G8" t="n">
-        <v>5.2</v>
+        <v>5.19</v>
       </c>
       <c r="H8" t="n">
-        <v>8630279.999999998</v>
+        <v>8601460</v>
       </c>
       <c r="I8" t="n">
         <v>6447</v>
@@ -1202,7 +1202,7 @@
         <v>3.68</v>
       </c>
       <c r="N8" t="n">
-        <v>8.85</v>
+        <v>8.84</v>
       </c>
       <c r="O8" t="n">
         <v>267.67</v>
@@ -1261,13 +1261,13 @@
         <v>2018</v>
       </c>
       <c r="B9" t="n">
-        <v>37.12</v>
+        <v>36.98</v>
       </c>
       <c r="C9" t="n">
-        <v>37.18</v>
+        <v>37.05</v>
       </c>
       <c r="D9" t="n">
-        <v>2.69</v>
+        <v>2.7</v>
       </c>
       <c r="E9" t="n">
         <v>1441</v>
@@ -1279,7 +1279,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>9946880</v>
+        <v>9910400</v>
       </c>
       <c r="I9" t="n">
         <v>6521</v>
@@ -1297,7 +1297,7 @@
         <v>-4.81</v>
       </c>
       <c r="N9" t="n">
-        <v>11.03</v>
+        <v>11</v>
       </c>
       <c r="O9" t="n">
         <v>-21.72</v>
@@ -1356,13 +1356,13 @@
         <v>2017</v>
       </c>
       <c r="B10" t="n">
-        <v>-3.45</v>
+        <v>-3.44</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>-28.97</v>
+        <v>-29.07</v>
       </c>
       <c r="E10" t="n">
         <v>469</v>
@@ -1371,10 +1371,10 @@
         <v>-20.26</v>
       </c>
       <c r="G10" t="n">
-        <v>3.77</v>
+        <v>3.76</v>
       </c>
       <c r="H10" t="n">
-        <v>7430480.000000001</v>
+        <v>7405120</v>
       </c>
       <c r="I10" t="n">
         <v>16404</v>
@@ -1392,7 +1392,7 @@
         <v>7.57</v>
       </c>
       <c r="N10" t="n">
-        <v>47.62</v>
+        <v>47.57</v>
       </c>
       <c r="O10" t="n">
         <v>-109.4</v>
@@ -1457,7 +1457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1614,949 +1614,949 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46112</v>
+        <v>46203</v>
       </c>
       <c r="B2" t="n">
-        <v>241.26</v>
+        <v>60.69</v>
       </c>
       <c r="C2" t="n">
-        <v>31.33</v>
+        <v>44.64</v>
       </c>
       <c r="D2" t="n">
-        <v>3.19</v>
+        <v>2.24</v>
       </c>
       <c r="E2" t="n">
-        <v>605</v>
+        <v>1301</v>
       </c>
       <c r="F2" t="n">
-        <v>1.22</v>
+        <v>6.76</v>
       </c>
       <c r="G2" t="n">
-        <v>6.19</v>
+        <v>6.33</v>
       </c>
       <c r="H2" t="n">
-        <v>30157830</v>
+        <v>30708940</v>
       </c>
       <c r="I2" t="n">
-        <v>23357</v>
+        <v>23467</v>
       </c>
       <c r="J2" t="n">
-        <v>235</v>
+        <v>212</v>
       </c>
       <c r="K2" t="n">
-        <v>23122</v>
+        <v>23255</v>
       </c>
       <c r="L2" t="n">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="M2" t="n">
-        <v>4.74</v>
+        <v>4.79</v>
       </c>
       <c r="N2" t="n">
-        <v>18.89</v>
+        <v>19.49</v>
       </c>
       <c r="O2" t="n">
-        <v>18.94</v>
+        <v>13.99</v>
       </c>
       <c r="P2" t="n">
-        <v>5.83</v>
+        <v>5.53</v>
       </c>
       <c r="Q2" t="n">
-        <v>-169</v>
+        <v>1117</v>
       </c>
       <c r="R2" t="n">
-        <v>-7072</v>
+        <v>-637</v>
       </c>
       <c r="S2" t="n">
-        <v>2652</v>
+        <v>-512</v>
       </c>
       <c r="T2" t="n">
-        <v>-486</v>
+        <v>779</v>
       </c>
       <c r="U2" t="n">
-        <v>317</v>
+        <v>338</v>
       </c>
       <c r="V2" t="n">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="W2" t="n">
         <v>0</v>
       </c>
       <c r="X2" t="n">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="Y2" t="n">
-        <v>-1925</v>
+        <v>-322</v>
       </c>
       <c r="Z2" t="n">
-        <v>27.83</v>
+        <v>11.43</v>
       </c>
       <c r="AA2" t="n">
-        <v>4864</v>
+        <v>4968</v>
       </c>
       <c r="AB2" t="n">
-        <v>1418</v>
+        <v>1132</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.65</v>
+        <v>0.47</v>
       </c>
       <c r="AD2" t="n">
-        <v>108</v>
+        <v>19.76</v>
       </c>
       <c r="AE2" t="n">
-        <v>481</v>
+        <v>450</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45930</v>
+        <v>46112</v>
       </c>
       <c r="B3" t="n">
-        <v>203.84</v>
+        <v>240.42</v>
       </c>
       <c r="C3" t="n">
-        <v>472.18</v>
+        <v>31.22</v>
       </c>
       <c r="D3" t="n">
-        <v>0.21</v>
+        <v>3.2</v>
       </c>
       <c r="E3" t="n">
-        <v>637</v>
+        <v>605</v>
       </c>
       <c r="F3" t="n">
-        <v>1.99</v>
+        <v>1.22</v>
       </c>
       <c r="G3" t="n">
-        <v>15.72</v>
+        <v>6.16</v>
       </c>
       <c r="H3" t="n">
-        <v>30984220</v>
+        <v>30052260</v>
       </c>
       <c r="I3" t="n">
-        <v>12111</v>
+        <v>23357</v>
       </c>
       <c r="J3" t="n">
-        <v>762</v>
+        <v>235</v>
       </c>
       <c r="K3" t="n">
-        <v>11349</v>
+        <v>23122</v>
       </c>
       <c r="L3" t="n">
-        <v>6.82</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="M3" t="n">
-        <v>5.76</v>
+        <v>4.74</v>
       </c>
       <c r="N3" t="n">
-        <v>25.44</v>
+        <v>18.86</v>
       </c>
       <c r="O3" t="n">
-        <v>1.57</v>
+        <v>18.94</v>
       </c>
       <c r="P3" t="n">
-        <v>5.05</v>
+        <v>5.83</v>
       </c>
       <c r="Q3" t="n">
-        <v>484</v>
+        <v>-169</v>
       </c>
       <c r="R3" t="n">
-        <v>-258</v>
+        <v>-7072</v>
       </c>
       <c r="S3" t="n">
-        <v>215</v>
+        <v>2652</v>
       </c>
       <c r="T3" t="n">
-        <v>816</v>
+        <v>-486</v>
       </c>
       <c r="U3" t="n">
-        <v>-332</v>
+        <v>317</v>
       </c>
       <c r="V3" t="n">
-        <v>36</v>
+        <v>222</v>
       </c>
       <c r="W3" t="n">
         <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>36</v>
+        <v>222</v>
       </c>
       <c r="Y3" t="n">
-        <v>411</v>
+        <v>-1925</v>
       </c>
       <c r="Z3" t="n">
-        <v>28.97</v>
+        <v>27.83</v>
       </c>
       <c r="AA3" t="n">
-        <v>890</v>
+        <v>4864</v>
       </c>
       <c r="AB3" t="n">
-        <v>264</v>
+        <v>1418</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.62</v>
+        <v>0.65</v>
       </c>
       <c r="AD3" t="n">
-        <v>78.29000000000001</v>
+        <v>108</v>
       </c>
       <c r="AE3" t="n">
-        <v>355</v>
+        <v>481</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45838</v>
+        <v>45930</v>
       </c>
       <c r="B4" t="n">
-        <v>-299.2</v>
+        <v>203.12</v>
       </c>
       <c r="C4" t="n">
-        <v>51.21</v>
+        <v>470.5</v>
       </c>
       <c r="D4" t="n">
-        <v>1.95</v>
+        <v>0.21</v>
       </c>
       <c r="E4" t="n">
-        <v>226</v>
+        <v>637</v>
       </c>
       <c r="F4" t="n">
-        <v>-1.54</v>
+        <v>1.99</v>
       </c>
       <c r="G4" t="n">
-        <v>13.6</v>
+        <v>15.67</v>
       </c>
       <c r="H4" t="n">
-        <v>31116960</v>
+        <v>30874210</v>
       </c>
       <c r="I4" t="n">
-        <v>11116</v>
+        <v>12111</v>
       </c>
       <c r="J4" t="n">
-        <v>197</v>
+        <v>762</v>
       </c>
       <c r="K4" t="n">
-        <v>10919</v>
+        <v>11349</v>
       </c>
       <c r="L4" t="n">
-        <v>4.01</v>
+        <v>6.82</v>
       </c>
       <c r="M4" t="n">
-        <v>4.77</v>
+        <v>5.76</v>
       </c>
       <c r="N4" t="n">
-        <v>15.44</v>
+        <v>25.37</v>
       </c>
       <c r="O4" t="n">
-        <v>26.97</v>
+        <v>1.57</v>
       </c>
       <c r="P4" t="n">
-        <v>11.03</v>
+        <v>5.05</v>
       </c>
       <c r="Q4" t="n">
-        <v>451</v>
+        <v>484</v>
       </c>
       <c r="R4" t="n">
-        <v>-948</v>
+        <v>-258</v>
       </c>
       <c r="S4" t="n">
-        <v>-297</v>
+        <v>215</v>
       </c>
       <c r="T4" t="n">
-        <v>-493</v>
+        <v>816</v>
       </c>
       <c r="U4" t="n">
-        <v>944</v>
+        <v>-332</v>
       </c>
       <c r="V4" t="n">
-        <v>419</v>
+        <v>36</v>
       </c>
       <c r="W4" t="n">
         <v>0</v>
       </c>
       <c r="X4" t="n">
-        <v>419</v>
+        <v>36</v>
       </c>
       <c r="Y4" t="n">
-        <v>-586</v>
+        <v>411</v>
       </c>
       <c r="Z4" t="n">
-        <v>23.94</v>
+        <v>28.97</v>
       </c>
       <c r="AA4" t="n">
-        <v>156</v>
+        <v>890</v>
       </c>
       <c r="AB4" t="n">
-        <v>823</v>
+        <v>264</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.44</v>
+        <v>0.62</v>
       </c>
       <c r="AD4" t="n">
-        <v>-82.69</v>
+        <v>78.29000000000001</v>
       </c>
       <c r="AE4" t="n">
-        <v>289</v>
+        <v>355</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45747</v>
+        <v>45838</v>
       </c>
       <c r="B5" t="n">
-        <v>24.82</v>
+        <v>-298.15</v>
       </c>
       <c r="C5" t="n">
-        <v>15.49</v>
+        <v>51.03</v>
       </c>
       <c r="D5" t="n">
-        <v>6.46</v>
+        <v>1.96</v>
       </c>
       <c r="E5" t="n">
-        <v>1352</v>
+        <v>226</v>
       </c>
       <c r="F5" t="n">
-        <v>8.74</v>
+        <v>-1.54</v>
       </c>
       <c r="G5" t="n">
-        <v>6.7</v>
+        <v>13.56</v>
       </c>
       <c r="H5" t="n">
-        <v>18612000</v>
+        <v>31007200</v>
       </c>
       <c r="I5" t="n">
-        <v>10986</v>
+        <v>11116</v>
       </c>
       <c r="J5" t="n">
-        <v>708</v>
+        <v>197</v>
       </c>
       <c r="K5" t="n">
-        <v>10278</v>
+        <v>10919</v>
       </c>
       <c r="L5" t="n">
-        <v>2.83</v>
+        <v>4.01</v>
       </c>
       <c r="M5" t="n">
-        <v>3.7</v>
+        <v>4.77</v>
       </c>
       <c r="N5" t="n">
-        <v>7.95</v>
+        <v>15.4</v>
       </c>
       <c r="O5" t="n">
-        <v>44.36</v>
+        <v>26.97</v>
       </c>
       <c r="P5" t="n">
-        <v>15.39</v>
+        <v>11.03</v>
       </c>
       <c r="Q5" t="n">
-        <v>855</v>
+        <v>451</v>
       </c>
       <c r="R5" t="n">
-        <v>-134</v>
+        <v>-948</v>
       </c>
       <c r="S5" t="n">
-        <v>-458</v>
+        <v>-297</v>
       </c>
       <c r="T5" t="n">
-        <v>618</v>
+        <v>-493</v>
       </c>
       <c r="U5" t="n">
-        <v>237</v>
+        <v>944</v>
       </c>
       <c r="V5" t="n">
-        <v>-476</v>
+        <v>419</v>
       </c>
       <c r="W5" t="n">
         <v>0</v>
       </c>
       <c r="X5" t="n">
-        <v>-476</v>
+        <v>419</v>
       </c>
       <c r="Y5" t="n">
-        <v>575</v>
+        <v>-586</v>
       </c>
       <c r="Z5" t="n">
-        <v>-10.53</v>
+        <v>23.94</v>
       </c>
       <c r="AA5" t="n">
-        <v>1091</v>
+        <v>156</v>
       </c>
       <c r="AB5" t="n">
-        <v>2206</v>
+        <v>823</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.61</v>
+        <v>0.44</v>
       </c>
       <c r="AD5" t="n">
-        <v>16.13</v>
+        <v>-82.69</v>
       </c>
       <c r="AE5" t="n">
-        <v>314</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45565</v>
+        <v>45747</v>
       </c>
       <c r="B6" t="n">
-        <v>-24</v>
+        <v>24.73</v>
       </c>
       <c r="C6" t="n">
-        <v>23.59</v>
+        <v>15.43</v>
       </c>
       <c r="D6" t="n">
-        <v>4.24</v>
+        <v>6.48</v>
       </c>
       <c r="E6" t="n">
-        <v>-551</v>
+        <v>1352</v>
       </c>
       <c r="F6" t="n">
-        <v>-10.62</v>
+        <v>8.74</v>
       </c>
       <c r="G6" t="n">
-        <v>7.31</v>
+        <v>6.68</v>
       </c>
       <c r="H6" t="n">
-        <v>18406440</v>
+        <v>18546660</v>
       </c>
       <c r="I6" t="n">
-        <v>10882</v>
+        <v>10986</v>
       </c>
       <c r="J6" t="n">
-        <v>1114</v>
+        <v>708</v>
       </c>
       <c r="K6" t="n">
-        <v>9768</v>
+        <v>10278</v>
       </c>
       <c r="L6" t="n">
-        <v>3.1</v>
+        <v>2.83</v>
       </c>
       <c r="M6" t="n">
-        <v>3.88</v>
+        <v>3.7</v>
       </c>
       <c r="N6" t="n">
-        <v>8.94</v>
+        <v>7.93</v>
       </c>
       <c r="O6" t="n">
-        <v>32.74</v>
+        <v>44.36</v>
       </c>
       <c r="P6" t="n">
-        <v>12.8</v>
+        <v>15.39</v>
       </c>
       <c r="Q6" t="n">
-        <v>31</v>
+        <v>855</v>
       </c>
       <c r="R6" t="n">
-        <v>364</v>
+        <v>-134</v>
       </c>
       <c r="S6" t="n">
-        <v>-350</v>
+        <v>-458</v>
       </c>
       <c r="T6" t="n">
-        <v>-84</v>
+        <v>618</v>
       </c>
       <c r="U6" t="n">
-        <v>115</v>
+        <v>237</v>
       </c>
       <c r="V6" t="n">
-        <v>-630</v>
+        <v>-476</v>
       </c>
       <c r="W6" t="n">
         <v>0</v>
       </c>
       <c r="X6" t="n">
-        <v>-630</v>
+        <v>-476</v>
       </c>
       <c r="Y6" t="n">
-        <v>1263</v>
+        <v>575</v>
       </c>
       <c r="Z6" t="n">
-        <v>-56.91</v>
+        <v>-10.53</v>
       </c>
       <c r="AA6" t="n">
-        <v>833</v>
+        <v>1091</v>
       </c>
       <c r="AB6" t="n">
-        <v>2512</v>
+        <v>2206</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.57</v>
+        <v>0.61</v>
       </c>
       <c r="AD6" t="n">
-        <v>-15.38</v>
+        <v>16.13</v>
       </c>
       <c r="AE6" t="n">
-        <v>226</v>
+        <v>314</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45473</v>
+        <v>45565</v>
       </c>
       <c r="B7" t="n">
-        <v>21.3</v>
+        <v>-23.91</v>
       </c>
       <c r="C7" t="n">
-        <v>8.58</v>
+        <v>23.5</v>
       </c>
       <c r="D7" t="n">
-        <v>11.66</v>
+        <v>4.25</v>
       </c>
       <c r="E7" t="n">
-        <v>1695</v>
+        <v>-551</v>
       </c>
       <c r="F7" t="n">
-        <v>11.08</v>
+        <v>-10.62</v>
       </c>
       <c r="G7" t="n">
-        <v>4.34</v>
+        <v>7.28</v>
       </c>
       <c r="H7" t="n">
-        <v>15720640</v>
+        <v>18342270</v>
       </c>
       <c r="I7" t="n">
-        <v>10922</v>
+        <v>10882</v>
       </c>
       <c r="J7" t="n">
-        <v>392</v>
+        <v>1114</v>
       </c>
       <c r="K7" t="n">
-        <v>10530</v>
+        <v>9768</v>
       </c>
       <c r="L7" t="n">
-        <v>2.31</v>
+        <v>3.1</v>
       </c>
       <c r="M7" t="n">
-        <v>2.91</v>
+        <v>3.88</v>
       </c>
       <c r="N7" t="n">
-        <v>5.77</v>
+        <v>8.92</v>
       </c>
       <c r="O7" t="n">
-        <v>52.44</v>
+        <v>32.74</v>
       </c>
       <c r="P7" t="n">
-        <v>18.71</v>
+        <v>12.8</v>
       </c>
       <c r="Q7" t="n">
-        <v>1056</v>
+        <v>31</v>
       </c>
       <c r="R7" t="n">
-        <v>-109</v>
+        <v>364</v>
       </c>
       <c r="S7" t="n">
-        <v>-403</v>
+        <v>-350</v>
       </c>
       <c r="T7" t="n">
-        <v>943</v>
+        <v>-84</v>
       </c>
       <c r="U7" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="V7" t="n">
-        <v>-611</v>
+        <v>-630</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>-611</v>
+        <v>-630</v>
       </c>
       <c r="Y7" t="n">
-        <v>1504</v>
+        <v>1263</v>
       </c>
       <c r="Z7" t="n">
-        <v>-12.53</v>
+        <v>-56.91</v>
       </c>
       <c r="AA7" t="n">
-        <v>994</v>
+        <v>833</v>
       </c>
       <c r="AB7" t="n">
-        <v>2707</v>
+        <v>2512</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.41</v>
+        <v>0.57</v>
       </c>
       <c r="AD7" t="n">
-        <v>11.65</v>
+        <v>-15.38</v>
       </c>
       <c r="AE7" t="n">
-        <v>90</v>
+        <v>226</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45382</v>
+        <v>45473</v>
       </c>
       <c r="B8" t="n">
-        <v>26.73</v>
+        <v>21.23</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.83</v>
+        <v>11.7</v>
       </c>
       <c r="E8" t="n">
-        <v>1140</v>
+        <v>1695</v>
       </c>
       <c r="F8" t="n">
-        <v>6.88</v>
+        <v>11.08</v>
       </c>
       <c r="G8" t="n">
-        <v>4.14</v>
+        <v>4.32</v>
       </c>
       <c r="H8" t="n">
-        <v>13658150</v>
+        <v>15666560</v>
       </c>
       <c r="I8" t="n">
-        <v>10878</v>
+        <v>10922</v>
       </c>
       <c r="J8" t="n">
-        <v>293</v>
+        <v>392</v>
       </c>
       <c r="K8" t="n">
-        <v>10585</v>
+        <v>10530</v>
       </c>
       <c r="L8" t="n">
-        <v>7.06</v>
+        <v>2.31</v>
       </c>
       <c r="M8" t="n">
-        <v>3.21</v>
+        <v>2.91</v>
       </c>
       <c r="N8" t="n">
-        <v>16.16</v>
+        <v>5.76</v>
       </c>
       <c r="O8" t="n">
-        <v>-5.25</v>
+        <v>52.44</v>
       </c>
       <c r="P8" t="n">
-        <v>2.94</v>
+        <v>18.71</v>
       </c>
       <c r="Q8" t="n">
-        <v>267</v>
+        <v>1056</v>
       </c>
       <c r="R8" t="n">
-        <v>-92</v>
+        <v>-109</v>
       </c>
       <c r="S8" t="n">
-        <v>-288</v>
+        <v>-403</v>
       </c>
       <c r="T8" t="n">
-        <v>176</v>
+        <v>943</v>
       </c>
       <c r="U8" t="n">
-        <v>91</v>
+        <v>113</v>
       </c>
       <c r="V8" t="n">
-        <v>2005</v>
+        <v>-611</v>
       </c>
       <c r="W8" t="n">
         <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>2005</v>
+        <v>-611</v>
       </c>
       <c r="Y8" t="n">
-        <v>92</v>
+        <v>1504</v>
       </c>
       <c r="Z8" t="n">
-        <v>666.67</v>
+        <v>-12.53</v>
       </c>
       <c r="AA8" t="n">
-        <v>-2121</v>
+        <v>994</v>
       </c>
       <c r="AB8" t="n">
-        <v>-2472</v>
+        <v>2707</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.41</v>
       </c>
       <c r="AD8" t="n">
-        <v>23.09</v>
+        <v>11.65</v>
       </c>
       <c r="AE8" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45199</v>
+        <v>45382</v>
       </c>
       <c r="B9" t="n">
-        <v>24.53</v>
+        <v>26.63</v>
       </c>
       <c r="C9" t="n">
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>-7.35</v>
+        <v>-0.83</v>
       </c>
       <c r="E9" t="n">
-        <v>869</v>
+        <v>1140</v>
       </c>
       <c r="F9" t="n">
-        <v>4.32</v>
+        <v>6.88</v>
       </c>
       <c r="G9" t="n">
-        <v>2.39</v>
+        <v>4.13</v>
       </c>
       <c r="H9" t="n">
-        <v>8413400</v>
+        <v>13610080</v>
       </c>
       <c r="I9" t="n">
-        <v>11900</v>
+        <v>10878</v>
       </c>
       <c r="J9" t="n">
-        <v>412</v>
+        <v>293</v>
       </c>
       <c r="K9" t="n">
-        <v>11488</v>
+        <v>10585</v>
       </c>
       <c r="L9" t="n">
-        <v>17.38</v>
+        <v>7.06</v>
       </c>
       <c r="M9" t="n">
-        <v>3.27</v>
+        <v>3.21</v>
       </c>
       <c r="N9" t="n">
-        <v>30.11</v>
+        <v>16.13</v>
       </c>
       <c r="O9" t="n">
-        <v>-17.54</v>
+        <v>-5.25</v>
       </c>
       <c r="P9" t="n">
-        <v>-0.85</v>
+        <v>2.94</v>
       </c>
       <c r="Q9" t="n">
-        <v>566</v>
+        <v>267</v>
       </c>
       <c r="R9" t="n">
-        <v>-129</v>
+        <v>-92</v>
       </c>
       <c r="S9" t="n">
-        <v>-572</v>
+        <v>-288</v>
       </c>
       <c r="T9" t="n">
-        <v>393</v>
+        <v>176</v>
       </c>
       <c r="U9" t="n">
-        <v>173</v>
+        <v>91</v>
       </c>
       <c r="V9" t="n">
-        <v>2144</v>
+        <v>2005</v>
       </c>
       <c r="W9" t="n">
         <v>0</v>
       </c>
       <c r="X9" t="n">
-        <v>2144</v>
+        <v>2005</v>
       </c>
       <c r="Y9" t="n">
-        <v>538</v>
+        <v>92</v>
       </c>
       <c r="Z9" t="n">
-        <v>-1803.05</v>
+        <v>666.67</v>
       </c>
       <c r="AA9" t="n">
-        <v>-1995</v>
+        <v>-2121</v>
       </c>
       <c r="AB9" t="n">
-        <v>-2659</v>
+        <v>-2472</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.53</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="AD9" t="n">
-        <v>35.28</v>
+        <v>23.09</v>
       </c>
       <c r="AE9" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45107</v>
+        <v>45199</v>
       </c>
       <c r="B10" t="n">
-        <v>26.36</v>
+        <v>24.44</v>
       </c>
       <c r="C10" t="n">
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>-5.75</v>
+        <v>-7.38</v>
       </c>
       <c r="E10" t="n">
-        <v>845</v>
+        <v>869</v>
       </c>
       <c r="F10" t="n">
-        <v>4.85</v>
+        <v>4.32</v>
       </c>
       <c r="G10" t="n">
-        <v>2.44</v>
+        <v>2.38</v>
       </c>
       <c r="H10" t="n">
-        <v>8119650</v>
+        <v>8383500</v>
       </c>
       <c r="I10" t="n">
-        <v>12312</v>
+        <v>11900</v>
       </c>
       <c r="J10" t="n">
-        <v>448</v>
+        <v>412</v>
       </c>
       <c r="K10" t="n">
-        <v>11864</v>
+        <v>11488</v>
       </c>
       <c r="L10" t="n">
-        <v>16.88</v>
+        <v>17.38</v>
       </c>
       <c r="M10" t="n">
-        <v>3.56</v>
+        <v>3.27</v>
       </c>
       <c r="N10" t="n">
-        <v>28.43</v>
+        <v>30.06</v>
       </c>
       <c r="O10" t="n">
-        <v>-13.42</v>
+        <v>-17.54</v>
       </c>
       <c r="P10" t="n">
-        <v>-0.16</v>
+        <v>-0.85</v>
       </c>
       <c r="Q10" t="n">
-        <v>570</v>
+        <v>566</v>
       </c>
       <c r="R10" t="n">
-        <v>-152</v>
+        <v>-129</v>
       </c>
       <c r="S10" t="n">
-        <v>-374</v>
+        <v>-572</v>
       </c>
       <c r="T10" t="n">
-        <v>382</v>
+        <v>393</v>
       </c>
       <c r="U10" t="n">
-        <v>188</v>
+        <v>173</v>
       </c>
       <c r="V10" t="n">
-        <v>2239</v>
+        <v>2144</v>
       </c>
       <c r="W10" t="n">
         <v>0</v>
       </c>
       <c r="X10" t="n">
-        <v>2239</v>
+        <v>2144</v>
       </c>
       <c r="Y10" t="n">
-        <v>245</v>
+        <v>538</v>
       </c>
       <c r="Z10" t="n">
-        <v>-9592</v>
+        <v>-1803.05</v>
       </c>
       <c r="AA10" t="n">
-        <v>-1250</v>
+        <v>-1995</v>
       </c>
       <c r="AB10" t="n">
-        <v>-2502</v>
+        <v>-2659</v>
       </c>
       <c r="AC10" t="n">
-        <v>0.38</v>
+        <v>0.53</v>
       </c>
       <c r="AD10" t="n">
-        <v>28.25</v>
+        <v>35.28</v>
       </c>
       <c r="AE10" t="n">
-        <v>8</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45016</v>
+        <v>45107</v>
       </c>
       <c r="B11" t="n">
-        <v>-5.49</v>
+        <v>26.27</v>
       </c>
       <c r="C11" t="n">
-        <v>8.35</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>11.98</v>
+        <v>-5.77</v>
       </c>
       <c r="E11" t="n">
-        <v>-1354</v>
+        <v>845</v>
       </c>
       <c r="F11" t="n">
-        <v>-17.29</v>
+        <v>4.85</v>
       </c>
       <c r="G11" t="n">
-        <v>2.38</v>
+        <v>2.43</v>
       </c>
       <c r="H11" t="n">
-        <v>7332400</v>
+        <v>8089620.000000001</v>
       </c>
       <c r="I11" t="n">
-        <v>12593</v>
+        <v>12312</v>
       </c>
       <c r="J11" t="n">
-        <v>439</v>
+        <v>448</v>
       </c>
       <c r="K11" t="n">
-        <v>12154</v>
+        <v>11864</v>
       </c>
       <c r="L11" t="n">
-        <v>4.93</v>
+        <v>16.88</v>
       </c>
       <c r="M11" t="n">
-        <v>3.95</v>
+        <v>3.56</v>
       </c>
       <c r="N11" t="n">
-        <v>7.9</v>
+        <v>28.38</v>
       </c>
       <c r="O11" t="n">
-        <v>31.85</v>
+        <v>-13.42</v>
       </c>
       <c r="P11" t="n">
-        <v>8.859999999999999</v>
+        <v>-0.16</v>
       </c>
       <c r="Q11" t="n">
-        <v>-1598</v>
+        <v>570</v>
       </c>
       <c r="R11" t="n">
-        <v>-2350</v>
+        <v>-152</v>
       </c>
       <c r="S11" t="n">
-        <v>2536</v>
+        <v>-374</v>
       </c>
       <c r="T11" t="n">
-        <v>-4232</v>
+        <v>382</v>
       </c>
       <c r="U11" t="n">
-        <v>2634</v>
+        <v>188</v>
       </c>
       <c r="V11" t="n">
-        <v>2269</v>
+        <v>2239</v>
       </c>
       <c r="W11" t="n">
         <v>0</v>
       </c>
       <c r="X11" t="n">
-        <v>2269</v>
+        <v>2239</v>
       </c>
       <c r="Y11" t="n">
-        <v>-118</v>
+        <v>245</v>
       </c>
       <c r="Z11" t="n">
-        <v>197.19</v>
+        <v>-9592</v>
       </c>
       <c r="AA11" t="n">
-        <v>123</v>
+        <v>-1250</v>
       </c>
       <c r="AB11" t="n">
-        <v>-1306</v>
+        <v>-2502</v>
       </c>
       <c r="AC11" t="n">
         <v>0.38</v>
       </c>
       <c r="AD11" t="n">
-        <v>-6.52</v>
+        <v>28.25</v>
       </c>
       <c r="AE11" t="n">
         <v>8</v>
@@ -2564,474 +2564,474 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>44834</v>
+        <v>45016</v>
       </c>
       <c r="B12" t="n">
-        <v>122.41</v>
+        <v>-5.47</v>
       </c>
       <c r="C12" t="n">
-        <v>2.15</v>
+        <v>8.31</v>
       </c>
       <c r="D12" t="n">
-        <v>46.48</v>
+        <v>12.03</v>
       </c>
       <c r="E12" t="n">
-        <v>301</v>
+        <v>-1354</v>
       </c>
       <c r="F12" t="n">
-        <v>0.79</v>
+        <v>-17.29</v>
       </c>
       <c r="G12" t="n">
-        <v>1.6</v>
+        <v>2.37</v>
       </c>
       <c r="H12" t="n">
-        <v>8201500</v>
+        <v>7304800</v>
       </c>
       <c r="I12" t="n">
-        <v>8315</v>
+        <v>12593</v>
       </c>
       <c r="J12" t="n">
-        <v>379</v>
+        <v>439</v>
       </c>
       <c r="K12" t="n">
-        <v>7936</v>
+        <v>12154</v>
       </c>
       <c r="L12" t="n">
-        <v>1.25</v>
+        <v>4.93</v>
       </c>
       <c r="M12" t="n">
-        <v>1.55</v>
+        <v>3.95</v>
       </c>
       <c r="N12" t="n">
-        <v>2.55</v>
+        <v>7.89</v>
       </c>
       <c r="O12" t="n">
-        <v>76.69</v>
+        <v>31.85</v>
       </c>
       <c r="P12" t="n">
-        <v>32.5</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="Q12" t="n">
-        <v>-1431</v>
+        <v>-1598</v>
       </c>
       <c r="R12" t="n">
-        <v>-86</v>
+        <v>-2350</v>
       </c>
       <c r="S12" t="n">
-        <v>441</v>
+        <v>2536</v>
       </c>
       <c r="T12" t="n">
-        <v>-1538</v>
+        <v>-4232</v>
       </c>
       <c r="U12" t="n">
-        <v>107</v>
+        <v>2634</v>
       </c>
       <c r="V12" t="n">
-        <v>-285</v>
+        <v>2269</v>
       </c>
       <c r="W12" t="n">
         <v>0</v>
       </c>
       <c r="X12" t="n">
-        <v>-285</v>
+        <v>2269</v>
       </c>
       <c r="Y12" t="n">
-        <v>4597</v>
+        <v>-118</v>
       </c>
       <c r="Z12" t="n">
-        <v>32.95</v>
+        <v>197.19</v>
       </c>
       <c r="AA12" t="n">
-        <v>2094</v>
+        <v>123</v>
       </c>
       <c r="AB12" t="n">
-        <v>3124</v>
+        <v>-1306</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.36</v>
+        <v>0.38</v>
       </c>
       <c r="AD12" t="n">
-        <v>125.37</v>
+        <v>-6.52</v>
       </c>
       <c r="AE12" t="n">
-        <v>118</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>44742</v>
+        <v>44834</v>
       </c>
       <c r="B13" t="n">
-        <v>15.93</v>
+        <v>121.99</v>
       </c>
       <c r="C13" t="n">
-        <v>1.7</v>
+        <v>2.14</v>
       </c>
       <c r="D13" t="n">
-        <v>58.96</v>
+        <v>46.64</v>
       </c>
       <c r="E13" t="n">
-        <v>911</v>
+        <v>301</v>
       </c>
       <c r="F13" t="n">
-        <v>7.04</v>
+        <v>0.79</v>
       </c>
       <c r="G13" t="n">
-        <v>1.54</v>
+        <v>1.59</v>
       </c>
       <c r="H13" t="n">
-        <v>8171759.999999999</v>
+        <v>8173300</v>
       </c>
       <c r="I13" t="n">
         <v>8315</v>
       </c>
       <c r="J13" t="n">
-        <v>624</v>
+        <v>379</v>
       </c>
       <c r="K13" t="n">
-        <v>7691</v>
+        <v>7936</v>
       </c>
       <c r="L13" t="n">
-        <v>1.01</v>
+        <v>1.25</v>
       </c>
       <c r="M13" t="n">
-        <v>1.45</v>
+        <v>1.55</v>
       </c>
       <c r="N13" t="n">
-        <v>2.07</v>
+        <v>2.54</v>
       </c>
       <c r="O13" t="n">
-        <v>93.3</v>
+        <v>76.69</v>
       </c>
       <c r="P13" t="n">
-        <v>39.71</v>
+        <v>32.5</v>
       </c>
       <c r="Q13" t="n">
-        <v>1513</v>
+        <v>-1431</v>
       </c>
       <c r="R13" t="n">
-        <v>-39</v>
+        <v>-86</v>
       </c>
       <c r="S13" t="n">
-        <v>127</v>
+        <v>441</v>
       </c>
       <c r="T13" t="n">
-        <v>1396</v>
+        <v>-1538</v>
       </c>
       <c r="U13" t="n">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="V13" t="n">
-        <v>-181</v>
+        <v>-285</v>
       </c>
       <c r="W13" t="n">
         <v>0</v>
       </c>
       <c r="X13" t="n">
-        <v>-181</v>
+        <v>-285</v>
       </c>
       <c r="Y13" t="n">
-        <v>4711</v>
+        <v>4597</v>
       </c>
       <c r="Z13" t="n">
-        <v>-3.27</v>
+        <v>32.95</v>
       </c>
       <c r="AA13" t="n">
-        <v>3972</v>
+        <v>2094</v>
       </c>
       <c r="AB13" t="n">
-        <v>5619</v>
+        <v>3124</v>
       </c>
       <c r="AC13" t="n">
-        <v>0.35</v>
+        <v>0.36</v>
       </c>
       <c r="AD13" t="n">
-        <v>16.18</v>
+        <v>125.37</v>
       </c>
       <c r="AE13" t="n">
-        <v>178</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>44651</v>
+        <v>44742</v>
       </c>
       <c r="B14" t="n">
-        <v>4.79</v>
+        <v>15.87</v>
       </c>
       <c r="C14" t="n">
-        <v>1.92</v>
+        <v>1.69</v>
       </c>
       <c r="D14" t="n">
-        <v>51.97</v>
+        <v>59.17</v>
       </c>
       <c r="E14" t="n">
-        <v>2608</v>
+        <v>911</v>
       </c>
       <c r="F14" t="n">
-        <v>21.99</v>
+        <v>7.04</v>
       </c>
       <c r="G14" t="n">
-        <v>1.65</v>
+        <v>1.54</v>
       </c>
       <c r="H14" t="n">
-        <v>8307859.999999999</v>
+        <v>8143320</v>
       </c>
       <c r="I14" t="n">
-        <v>8332</v>
+        <v>8315</v>
       </c>
       <c r="J14" t="n">
-        <v>426</v>
+        <v>624</v>
       </c>
       <c r="K14" t="n">
-        <v>7906</v>
+        <v>7691</v>
       </c>
       <c r="L14" t="n">
-        <v>1.13</v>
+        <v>1.01</v>
       </c>
       <c r="M14" t="n">
-        <v>1.57</v>
+        <v>1.45</v>
       </c>
       <c r="N14" t="n">
-        <v>2.32</v>
+        <v>2.07</v>
       </c>
       <c r="O14" t="n">
-        <v>86.48</v>
+        <v>93.3</v>
       </c>
       <c r="P14" t="n">
-        <v>36.18</v>
+        <v>39.71</v>
       </c>
       <c r="Q14" t="n">
-        <v>1676</v>
+        <v>1513</v>
       </c>
       <c r="R14" t="n">
-        <v>-80</v>
+        <v>-39</v>
       </c>
       <c r="S14" t="n">
-        <v>287</v>
+        <v>127</v>
       </c>
       <c r="T14" t="n">
-        <v>1590</v>
+        <v>1396</v>
       </c>
       <c r="U14" t="n">
-        <v>86</v>
+        <v>117</v>
       </c>
       <c r="V14" t="n">
-        <v>3087</v>
+        <v>-181</v>
       </c>
       <c r="W14" t="n">
         <v>0</v>
       </c>
       <c r="X14" t="n">
-        <v>3087</v>
+        <v>-181</v>
       </c>
       <c r="Y14" t="n">
-        <v>4604</v>
+        <v>4711</v>
       </c>
       <c r="Z14" t="n">
-        <v>73.22999999999999</v>
+        <v>-3.27</v>
       </c>
       <c r="AA14" t="n">
-        <v>483</v>
+        <v>3972</v>
       </c>
       <c r="AB14" t="n">
-        <v>1159</v>
+        <v>5619</v>
       </c>
       <c r="AC14" t="n">
         <v>0.35</v>
       </c>
       <c r="AD14" t="n">
-        <v>4.9</v>
+        <v>16.18</v>
       </c>
       <c r="AE14" t="n">
-        <v>188</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>44469</v>
+        <v>44651</v>
       </c>
       <c r="B15" t="n">
-        <v>5.44</v>
+        <v>4.77</v>
       </c>
       <c r="C15" t="n">
-        <v>3.07</v>
+        <v>1.92</v>
       </c>
       <c r="D15" t="n">
-        <v>32.54</v>
+        <v>52.15</v>
       </c>
       <c r="E15" t="n">
-        <v>2518</v>
+        <v>2608</v>
       </c>
       <c r="F15" t="n">
-        <v>24.48</v>
+        <v>21.99</v>
       </c>
       <c r="G15" t="n">
-        <v>2.16</v>
+        <v>1.65</v>
       </c>
       <c r="H15" t="n">
-        <v>8802850</v>
+        <v>8278820</v>
       </c>
       <c r="I15" t="n">
-        <v>8797</v>
+        <v>8332</v>
       </c>
       <c r="J15" t="n">
-        <v>273</v>
+        <v>426</v>
       </c>
       <c r="K15" t="n">
-        <v>8524</v>
+        <v>7906</v>
       </c>
       <c r="L15" t="n">
-        <v>1.75</v>
+        <v>1.13</v>
       </c>
       <c r="M15" t="n">
-        <v>2.09</v>
+        <v>1.57</v>
       </c>
       <c r="N15" t="n">
-        <v>3.55</v>
+        <v>2.31</v>
       </c>
       <c r="O15" t="n">
-        <v>70.20999999999999</v>
+        <v>86.48</v>
       </c>
       <c r="P15" t="n">
-        <v>25.48</v>
+        <v>36.18</v>
       </c>
       <c r="Q15" t="n">
-        <v>1478</v>
+        <v>1676</v>
       </c>
       <c r="R15" t="n">
-        <v>-93</v>
+        <v>-80</v>
       </c>
       <c r="S15" t="n">
-        <v>-270</v>
+        <v>287</v>
       </c>
       <c r="T15" t="n">
-        <v>1389</v>
+        <v>1590</v>
       </c>
       <c r="U15" t="n">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="V15" t="n">
-        <v>3413</v>
+        <v>3087</v>
       </c>
       <c r="W15" t="n">
         <v>0</v>
       </c>
       <c r="X15" t="n">
-        <v>3414</v>
+        <v>3087</v>
       </c>
       <c r="Y15" t="n">
-        <v>2563</v>
+        <v>4604</v>
       </c>
       <c r="Z15" t="n">
-        <v>119.23</v>
+        <v>73.22999999999999</v>
       </c>
       <c r="AA15" t="n">
-        <v>-1398</v>
+        <v>483</v>
       </c>
       <c r="AB15" t="n">
-        <v>-760</v>
+        <v>1159</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.33</v>
+        <v>0.35</v>
       </c>
       <c r="AD15" t="n">
-        <v>4.94</v>
+        <v>4.9</v>
       </c>
       <c r="AE15" t="n">
-        <v>0</v>
+        <v>188</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>44377</v>
+        <v>44469</v>
       </c>
       <c r="B16" t="n">
-        <v>8</v>
+        <v>5.42</v>
       </c>
       <c r="C16" t="n">
-        <v>5.52</v>
+        <v>3.06</v>
       </c>
       <c r="D16" t="n">
-        <v>18.1</v>
+        <v>32.65</v>
       </c>
       <c r="E16" t="n">
-        <v>1610</v>
+        <v>2518</v>
       </c>
       <c r="F16" t="n">
-        <v>20.56</v>
+        <v>24.48</v>
       </c>
       <c r="G16" t="n">
-        <v>3.39</v>
+        <v>2.15</v>
       </c>
       <c r="H16" t="n">
-        <v>8621550</v>
+        <v>8771000</v>
       </c>
       <c r="I16" t="n">
-        <v>9142</v>
+        <v>8797</v>
       </c>
       <c r="J16" t="n">
-        <v>376</v>
+        <v>273</v>
       </c>
       <c r="K16" t="n">
-        <v>8766</v>
+        <v>8524</v>
       </c>
       <c r="L16" t="n">
-        <v>2.96</v>
+        <v>1.75</v>
       </c>
       <c r="M16" t="n">
-        <v>3.45</v>
+        <v>2.09</v>
       </c>
       <c r="N16" t="n">
-        <v>5.88</v>
+        <v>3.54</v>
       </c>
       <c r="O16" t="n">
-        <v>61.24</v>
+        <v>70.20999999999999</v>
       </c>
       <c r="P16" t="n">
-        <v>16.17</v>
+        <v>25.48</v>
       </c>
       <c r="Q16" t="n">
-        <v>1294</v>
+        <v>1478</v>
       </c>
       <c r="R16" t="n">
-        <v>-128</v>
+        <v>-93</v>
       </c>
       <c r="S16" t="n">
-        <v>-831</v>
+        <v>-270</v>
       </c>
       <c r="T16" t="n">
-        <v>1175</v>
+        <v>1389</v>
       </c>
       <c r="U16" t="n">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="V16" t="n">
-        <v>3463</v>
+        <v>3413</v>
       </c>
       <c r="W16" t="n">
         <v>0</v>
       </c>
       <c r="X16" t="n">
-        <v>3466</v>
+        <v>3414</v>
       </c>
       <c r="Y16" t="n">
-        <v>1693</v>
+        <v>2563</v>
       </c>
       <c r="Z16" t="n">
-        <v>200.69</v>
+        <v>119.23</v>
       </c>
       <c r="AA16" t="n">
-        <v>-2824</v>
+        <v>-1398</v>
       </c>
       <c r="AB16" t="n">
-        <v>-2032</v>
+        <v>-760</v>
       </c>
       <c r="AC16" t="n">
-        <v>0.32</v>
+        <v>0.33</v>
       </c>
       <c r="AD16" t="n">
-        <v>7.33</v>
+        <v>4.94</v>
       </c>
       <c r="AE16" t="n">
         <v>0</v>
@@ -3039,96 +3039,191 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
+        <v>44377</v>
+      </c>
+      <c r="B17" t="n">
+        <v>7.97</v>
+      </c>
+      <c r="C17" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D17" t="n">
+        <v>18.17</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1610</v>
+      </c>
+      <c r="F17" t="n">
+        <v>20.56</v>
+      </c>
+      <c r="G17" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="H17" t="n">
+        <v>8589700</v>
+      </c>
+      <c r="I17" t="n">
+        <v>9142</v>
+      </c>
+      <c r="J17" t="n">
+        <v>376</v>
+      </c>
+      <c r="K17" t="n">
+        <v>8766</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="M17" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="N17" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="O17" t="n">
+        <v>61.24</v>
+      </c>
+      <c r="P17" t="n">
+        <v>16.17</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>1294</v>
+      </c>
+      <c r="R17" t="n">
+        <v>-128</v>
+      </c>
+      <c r="S17" t="n">
+        <v>-831</v>
+      </c>
+      <c r="T17" t="n">
+        <v>1175</v>
+      </c>
+      <c r="U17" t="n">
+        <v>119</v>
+      </c>
+      <c r="V17" t="n">
+        <v>3463</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" t="n">
+        <v>3466</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>1693</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>200.69</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>-2824</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>-2032</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
         <v>44286</v>
       </c>
-      <c r="B17" t="n">
-        <v>-97.55</v>
-      </c>
-      <c r="C17" t="n">
-        <v>13.27</v>
-      </c>
-      <c r="D17" t="n">
-        <v>7.53</v>
-      </c>
-      <c r="E17" t="n">
+      <c r="B18" t="n">
+        <v>-97.19</v>
+      </c>
+      <c r="C18" t="n">
+        <v>13.22</v>
+      </c>
+      <c r="D18" t="n">
+        <v>7.56</v>
+      </c>
+      <c r="E18" t="n">
         <v>261</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" t="n">
         <v>-1.01</v>
       </c>
-      <c r="G17" t="n">
-        <v>5.27</v>
-      </c>
-      <c r="H17" t="n">
-        <v>7999250</v>
-      </c>
-      <c r="I17" t="n">
+      <c r="G18" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="H18" t="n">
+        <v>7969850</v>
+      </c>
+      <c r="I18" t="n">
         <v>9895</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J18" t="n">
         <v>519</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K18" t="n">
         <v>9376</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L18" t="n">
         <v>5.52</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M18" t="n">
         <v>6.18</v>
       </c>
-      <c r="N17" t="n">
-        <v>10.22</v>
-      </c>
-      <c r="O17" t="n">
+      <c r="N18" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="O18" t="n">
         <v>39.62</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P18" t="n">
         <v>8.18</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="Q18" t="n">
         <v>-917</v>
       </c>
-      <c r="R17" t="n">
+      <c r="R18" t="n">
         <v>-3364</v>
       </c>
-      <c r="S17" t="n">
+      <c r="S18" t="n">
         <v>924</v>
       </c>
-      <c r="T17" t="n">
+      <c r="T18" t="n">
         <v>-4462</v>
       </c>
-      <c r="U17" t="n">
+      <c r="U18" t="n">
         <v>3545</v>
       </c>
-      <c r="V17" t="n">
+      <c r="V18" t="n">
         <v>3354</v>
       </c>
-      <c r="W17" t="n">
-        <v>0</v>
-      </c>
-      <c r="X17" t="n">
+      <c r="W18" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" t="n">
         <v>3360</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="Y18" t="n">
         <v>757</v>
       </c>
-      <c r="Z17" t="n">
+      <c r="Z18" t="n">
         <v>554.0700000000001</v>
       </c>
-      <c r="AA17" t="n">
+      <c r="AA18" t="n">
         <v>-3856</v>
       </c>
-      <c r="AB17" t="n">
+      <c r="AB18" t="n">
         <v>-4646</v>
       </c>
-      <c r="AC17" t="n">
+      <c r="AC18" t="n">
         <v>0.33</v>
       </c>
-      <c r="AD17" t="n">
+      <c r="AD18" t="n">
         <v>-97.56</v>
       </c>
-      <c r="AE17" t="n">
+      <c r="AE18" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>